<commit_message>
Aggiunto test 38 accreditamento medical-live
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MUREXSOFTWARESRLXX/Murex_Software_srl/medical-live/1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MUREXSOFTWARESRLXX/Murex_Software_srl/medical-live/1.0/report-checklist.xlsx
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="453">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1758,6 +1758,9 @@
   </si>
   <si>
     <t>Test non eseguito (timeout non simulato in ambiente di validazione)</t>
+  </si>
+  <si>
+    <t>f39457ebe1a7fc58577aae49fa941b19</t>
   </si>
 </sst>
 </file>
@@ -3822,10 +3825,10 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns6="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:W750"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
     <col min="2" max="2" width="46.85546875" customWidth="1"/>
@@ -3842,7 +3845,7 @@
     <col min="27" max="27" width="30.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="C1" s="4"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
@@ -3863,7 +3866,7 @@
       <c r="V1" s="2"/>
       <c r="W1" s="9"/>
     </row>
-    <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A2" s="50" t="s">
         <v>12</v>
       </c>
@@ -3891,7 +3894,7 @@
       <c r="V2" s="2"/>
       <c r="W2" s="9"/>
     </row>
-    <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A3" s="53" t="s">
         <v>13</v>
       </c>
@@ -3919,7 +3922,7 @@
       <c r="V3" s="2"/>
       <c r="W3" s="9"/>
     </row>
-    <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A4" s="55"/>
       <c r="B4" s="56"/>
       <c r="C4" s="59" t="s">
@@ -3946,7 +3949,7 @@
       <c r="V4" s="2"/>
       <c r="W4" s="9"/>
     </row>
-    <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A5" s="57"/>
       <c r="B5" s="58"/>
       <c r="C5" s="59" t="s">
@@ -3972,7 +3975,7 @@
       <c r="V5" s="2"/>
       <c r="W5" s="9"/>
     </row>
-    <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A6" s="48"/>
       <c r="B6" s="49"/>
       <c r="C6" s="10"/>
@@ -3995,7 +3998,7 @@
       <c r="V6" s="2"/>
       <c r="W6" s="9"/>
     </row>
-    <row r="7" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -4018,7 +4021,7 @@
       <c r="V7" s="2"/>
       <c r="W7" s="9"/>
     </row>
-    <row r="8" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" ht="14.25" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -4038,7 +4041,7 @@
       <c r="V8" s="2"/>
       <c r="W8" s="9"/>
     </row>
-    <row r="9" spans="1:23" s="18" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" s="18" customFormat="1" ht="14.25" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A9" s="19" t="s">
         <v>14</v>
       </c>
@@ -4109,7 +4112,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A10" s="33">
         <v>4</v>
       </c>
@@ -4146,7 +4149,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A11" s="35">
         <v>28</v>
       </c>
@@ -4183,7 +4186,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A12" s="35">
         <v>29</v>
       </c>
@@ -4220,7 +4223,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A13" s="35">
         <v>30</v>
       </c>
@@ -4261,7 +4264,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A14" s="35">
         <v>31</v>
       </c>
@@ -4298,7 +4301,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A15" s="35">
         <v>32</v>
       </c>
@@ -4335,7 +4338,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A16" s="35">
         <v>33</v>
       </c>
@@ -4372,7 +4375,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A17" s="35">
         <v>34</v>
       </c>
@@ -4409,7 +4412,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A18" s="35">
         <v>35</v>
       </c>
@@ -4446,7 +4449,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A19" s="35">
         <v>36</v>
       </c>
@@ -4483,7 +4486,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A20" s="35">
         <v>37</v>
       </c>
@@ -4520,7 +4523,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A21" s="35">
         <v>38</v>
       </c>
@@ -4537,13 +4540,13 @@
         <v>55</v>
       </c>
       <c r="F21" s="37">
-        <v>46079</v>
+        <v>46245</v>
       </c>
       <c r="G21" s="47">
-        <v>46079.695138888892</v>
+        <v>46245.43528935185</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="I21" s="42" t="s">
         <v>446</v>
@@ -4587,7 +4590,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A22" s="35">
         <v>39</v>
       </c>
@@ -4624,7 +4627,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A23" s="35">
         <v>40</v>
       </c>
@@ -4661,7 +4664,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A24" s="35">
         <v>41</v>
       </c>
@@ -4698,7 +4701,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A25" s="35">
         <v>42</v>
       </c>
@@ -4735,7 +4738,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A26" s="35">
         <v>43</v>
       </c>
@@ -4772,7 +4775,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A27" s="35">
         <v>44</v>
       </c>
@@ -4811,7 +4814,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A28" s="35">
         <v>45</v>
       </c>
@@ -4850,7 +4853,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A29" s="35">
         <v>46</v>
       </c>
@@ -4905,7 +4908,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A30" s="35">
         <v>47</v>
       </c>
@@ -4944,7 +4947,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A31" s="35">
         <v>48</v>
       </c>
@@ -4983,7 +4986,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A32" s="35">
         <v>49</v>
       </c>
@@ -5022,7 +5025,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A33" s="35">
         <v>50</v>
       </c>
@@ -5061,7 +5064,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A34" s="35">
         <v>51</v>
       </c>
@@ -5100,7 +5103,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A35" s="35">
         <v>53</v>
       </c>
@@ -5137,7 +5140,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A36" s="35">
         <v>55</v>
       </c>
@@ -5174,7 +5177,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A37" s="35">
         <v>56</v>
       </c>
@@ -5211,7 +5214,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A38" s="35">
         <v>57</v>
       </c>
@@ -5248,7 +5251,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A39" s="35">
         <v>59</v>
       </c>
@@ -5285,7 +5288,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A40" s="35">
         <v>60</v>
       </c>
@@ -5322,7 +5325,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A41" s="35">
         <v>61</v>
       </c>
@@ -5359,7 +5362,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A42" s="35">
         <v>62</v>
       </c>
@@ -5396,7 +5399,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A43" s="35">
         <v>64</v>
       </c>
@@ -5433,7 +5436,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A44" s="35">
         <v>66</v>
       </c>
@@ -5470,7 +5473,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A45" s="35">
         <v>67</v>
       </c>
@@ -5507,7 +5510,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A46" s="35">
         <v>68</v>
       </c>
@@ -5544,7 +5547,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A47" s="35">
         <v>69</v>
       </c>
@@ -5581,7 +5584,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A48" s="35">
         <v>70</v>
       </c>
@@ -5618,7 +5621,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A49" s="35">
         <v>71</v>
       </c>
@@ -5655,7 +5658,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A50" s="35">
         <v>72</v>
       </c>
@@ -5692,7 +5695,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A51" s="35">
         <v>73</v>
       </c>
@@ -5729,7 +5732,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A52" s="35">
         <v>74</v>
       </c>
@@ -5766,7 +5769,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A53" s="35">
         <v>76</v>
       </c>
@@ -5803,7 +5806,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A54" s="35">
         <v>78</v>
       </c>
@@ -5840,7 +5843,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A55" s="35">
         <v>79</v>
       </c>
@@ -5877,7 +5880,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A56" s="35">
         <v>80</v>
       </c>
@@ -5914,7 +5917,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A57" s="35">
         <v>81</v>
       </c>
@@ -5951,7 +5954,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A58" s="35">
         <v>83</v>
       </c>
@@ -5988,7 +5991,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A59" s="35">
         <v>84</v>
       </c>
@@ -6025,7 +6028,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A60" s="35">
         <v>85</v>
       </c>
@@ -6062,7 +6065,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A61" s="35">
         <v>86</v>
       </c>
@@ -6099,7 +6102,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A62" s="35">
         <v>87</v>
       </c>
@@ -6136,7 +6139,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A63" s="35">
         <v>88</v>
       </c>
@@ -6173,7 +6176,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A64" s="35">
         <v>89</v>
       </c>
@@ -6210,7 +6213,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A65" s="35">
         <v>90</v>
       </c>
@@ -6247,7 +6250,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A66" s="35">
         <v>91</v>
       </c>
@@ -6284,7 +6287,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A67" s="35">
         <v>92</v>
       </c>
@@ -6321,7 +6324,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A68" s="35">
         <v>93</v>
       </c>
@@ -6358,7 +6361,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A69" s="35">
         <v>95</v>
       </c>
@@ -6395,7 +6398,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A70" s="35">
         <v>97</v>
       </c>
@@ -6432,7 +6435,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A71" s="35">
         <v>98</v>
       </c>
@@ -6469,7 +6472,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A72" s="35">
         <v>99</v>
       </c>
@@ -6506,7 +6509,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A73" s="35">
         <v>100</v>
       </c>
@@ -6543,7 +6546,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A74" s="35">
         <v>101</v>
       </c>
@@ -6580,7 +6583,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A75" s="35">
         <v>102</v>
       </c>
@@ -6617,7 +6620,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A76" s="35">
         <v>103</v>
       </c>
@@ -6654,7 +6657,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A77" s="35">
         <v>104</v>
       </c>
@@ -6691,7 +6694,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A78" s="35">
         <v>105</v>
       </c>
@@ -6728,7 +6731,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A79" s="35">
         <v>106</v>
       </c>
@@ -6765,7 +6768,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A80" s="35">
         <v>108</v>
       </c>
@@ -6802,7 +6805,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A81" s="35">
         <v>110</v>
       </c>
@@ -6839,7 +6842,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A82" s="35">
         <v>111</v>
       </c>
@@ -6876,7 +6879,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A83" s="35">
         <v>112</v>
       </c>
@@ -6913,7 +6916,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A84" s="35">
         <v>113</v>
       </c>
@@ -6950,7 +6953,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A85" s="35">
         <v>114</v>
       </c>
@@ -6987,7 +6990,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A86" s="35">
         <v>115</v>
       </c>
@@ -7024,7 +7027,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A87" s="35">
         <v>116</v>
       </c>
@@ -7061,7 +7064,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A88" s="35">
         <v>117</v>
       </c>
@@ -7098,7 +7101,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A89" s="35">
         <v>118</v>
       </c>
@@ -7135,7 +7138,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A90" s="35">
         <v>119</v>
       </c>
@@ -7172,7 +7175,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A91" s="35">
         <v>120</v>
       </c>
@@ -7209,7 +7212,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A92" s="35">
         <v>121</v>
       </c>
@@ -7246,7 +7249,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A93" s="35">
         <v>123</v>
       </c>
@@ -7283,7 +7286,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A94" s="35">
         <v>125</v>
       </c>
@@ -7320,7 +7323,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A95" s="35">
         <v>126</v>
       </c>
@@ -7357,7 +7360,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A96" s="35">
         <v>127</v>
       </c>
@@ -7394,7 +7397,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A97" s="35">
         <v>128</v>
       </c>
@@ -7431,7 +7434,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A98" s="35">
         <v>129</v>
       </c>
@@ -7468,7 +7471,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A99" s="35">
         <v>130</v>
       </c>
@@ -7505,7 +7508,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A100" s="35">
         <v>131</v>
       </c>
@@ -7542,7 +7545,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A101" s="35">
         <v>132</v>
       </c>
@@ -7579,7 +7582,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A102" s="35">
         <v>133</v>
       </c>
@@ -7616,7 +7619,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A103" s="35">
         <v>134</v>
       </c>
@@ -7653,7 +7656,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A104" s="35">
         <v>135</v>
       </c>
@@ -7690,7 +7693,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A105" s="35">
         <v>136</v>
       </c>
@@ -7727,7 +7730,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A106" s="35">
         <v>137</v>
       </c>
@@ -7764,7 +7767,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A107" s="35">
         <v>138</v>
       </c>
@@ -7801,7 +7804,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A108" s="35">
         <v>139</v>
       </c>
@@ -7838,7 +7841,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A109" s="35">
         <v>140</v>
       </c>
@@ -7875,7 +7878,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A110" s="35">
         <v>141</v>
       </c>
@@ -7912,7 +7915,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A111" s="35">
         <v>142</v>
       </c>
@@ -7949,7 +7952,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A112" s="35">
         <v>143</v>
       </c>
@@ -7986,7 +7989,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A113" s="35">
         <v>144</v>
       </c>
@@ -8023,7 +8026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A114" s="35">
         <v>145</v>
       </c>
@@ -8060,7 +8063,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A115" s="35">
         <v>146</v>
       </c>
@@ -8097,7 +8100,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A116" s="35">
         <v>152</v>
       </c>
@@ -8134,7 +8137,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A117" s="35">
         <v>154</v>
       </c>
@@ -8171,7 +8174,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A118" s="35">
         <v>155</v>
       </c>
@@ -8208,7 +8211,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A119" s="35">
         <v>156</v>
       </c>
@@ -8245,7 +8248,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A120" s="35">
         <v>159</v>
       </c>
@@ -8282,7 +8285,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A121" s="35">
         <v>160</v>
       </c>
@@ -8319,7 +8322,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A122" s="35">
         <v>161</v>
       </c>
@@ -8356,7 +8359,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A123" s="35">
         <v>162</v>
       </c>
@@ -8393,7 +8396,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A124" s="35">
         <v>163</v>
       </c>
@@ -8430,7 +8433,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A125" s="35">
         <v>164</v>
       </c>
@@ -8467,7 +8470,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A126" s="35">
         <v>165</v>
       </c>
@@ -8504,7 +8507,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A127" s="35">
         <v>166</v>
       </c>
@@ -8541,7 +8544,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A128" s="35">
         <v>167</v>
       </c>
@@ -8578,7 +8581,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A129" s="35">
         <v>168</v>
       </c>
@@ -8615,7 +8618,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A130" s="35">
         <v>169</v>
       </c>
@@ -8652,7 +8655,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A131" s="35">
         <v>175</v>
       </c>
@@ -8693,7 +8696,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A132" s="35">
         <v>177</v>
       </c>
@@ -8734,7 +8737,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A133" s="35">
         <v>178</v>
       </c>
@@ -8775,7 +8778,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A134" s="35">
         <v>179</v>
       </c>
@@ -8816,7 +8819,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A135" s="35">
         <v>180</v>
       </c>
@@ -8857,7 +8860,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A136" s="35">
         <v>181</v>
       </c>
@@ -8898,7 +8901,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A137" s="35">
         <v>182</v>
       </c>
@@ -8939,7 +8942,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A138" s="35">
         <v>183</v>
       </c>
@@ -8980,7 +8983,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A139" s="35">
         <v>184</v>
       </c>
@@ -9021,7 +9024,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A140" s="35">
         <v>185</v>
       </c>
@@ -9062,7 +9065,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A141" s="35">
         <v>186</v>
       </c>
@@ -9103,7 +9106,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A142" s="35">
         <v>187</v>
       </c>
@@ -9144,7 +9147,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A143" s="35">
         <v>188</v>
       </c>
@@ -9185,7 +9188,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A144" s="35">
         <v>189</v>
       </c>
@@ -9226,7 +9229,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A145" s="35">
         <v>190</v>
       </c>
@@ -9267,7 +9270,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A146" s="35">
         <v>191</v>
       </c>
@@ -9304,7 +9307,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A147" s="35">
         <v>376</v>
       </c>
@@ -9341,7 +9344,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A148" s="35">
         <v>417</v>
       </c>
@@ -9378,7 +9381,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A149" s="35">
         <v>418</v>
       </c>
@@ -9415,7 +9418,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A150" s="35">
         <v>419</v>
       </c>
@@ -9452,7 +9455,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A151" s="35">
         <v>423</v>
       </c>
@@ -9489,7 +9492,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A152" s="35">
         <v>424</v>
       </c>
@@ -9526,7 +9529,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A153" s="35">
         <v>425</v>
       </c>
@@ -9563,7 +9566,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A154" s="35">
         <v>432</v>
       </c>
@@ -9600,7 +9603,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A155" s="35">
         <v>433</v>
       </c>
@@ -9637,7 +9640,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A156" s="35">
         <v>434</v>
       </c>
@@ -9674,7 +9677,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A157" s="35">
         <v>435</v>
       </c>
@@ -9711,7 +9714,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A158" s="35">
         <v>437</v>
       </c>
@@ -9748,7 +9751,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A159" s="35">
         <v>438</v>
       </c>
@@ -9785,7 +9788,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A160" s="35">
         <v>440</v>
       </c>
@@ -9822,7 +9825,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A161" s="35">
         <v>441</v>
       </c>
@@ -9859,7 +9862,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A162" s="35">
         <v>442</v>
       </c>
@@ -9896,7 +9899,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A163" s="35">
         <v>443</v>
       </c>
@@ -9933,7 +9936,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A164" s="35">
         <v>448</v>
       </c>
@@ -9970,7 +9973,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A165" s="35">
         <v>449</v>
       </c>
@@ -10007,7 +10010,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A166" s="35">
         <v>450</v>
       </c>
@@ -10044,7 +10047,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A167" s="35">
         <v>451</v>
       </c>
@@ -10081,7 +10084,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A168" s="35">
         <v>452</v>
       </c>
@@ -10118,7 +10121,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A169" s="35">
         <v>454</v>
       </c>
@@ -10155,7 +10158,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A170" s="35">
         <v>455</v>
       </c>
@@ -10192,7 +10195,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A171" s="35">
         <v>456</v>
       </c>
@@ -10229,7 +10232,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A172" s="35">
         <v>457</v>
       </c>
@@ -10266,7 +10269,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A173" s="35">
         <v>458</v>
       </c>
@@ -10303,7 +10306,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A174" s="35">
         <v>459</v>
       </c>
@@ -10340,7 +10343,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A175" s="35">
         <v>460</v>
       </c>
@@ -10377,7 +10380,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A176" s="35">
         <v>461</v>
       </c>
@@ -10414,7 +10417,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A177" s="35">
         <v>462</v>
       </c>
@@ -10451,7 +10454,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A178" s="35">
         <v>463</v>
       </c>
@@ -10488,7 +10491,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A179" s="35">
         <v>464</v>
       </c>
@@ -10525,7 +10528,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A180" s="35">
         <v>465</v>
       </c>
@@ -10562,7 +10565,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A181" s="35">
         <v>466</v>
       </c>
@@ -10599,7 +10602,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A182" s="35">
         <v>467</v>
       </c>
@@ -10636,7 +10639,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A183" s="35">
         <v>468</v>
       </c>
@@ -10673,7 +10676,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:23" ht="14.25" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A184" s="35">
         <v>469</v>
       </c>
@@ -10714,7 +10717,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A185" s="35">
         <v>470</v>
       </c>
@@ -10751,7 +10754,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A186" s="35">
         <v>471</v>
       </c>
@@ -10788,7 +10791,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A187" s="35">
         <v>472</v>
       </c>
@@ -10825,7 +10828,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A188" s="35">
         <v>473</v>
       </c>
@@ -10862,7 +10865,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A189" s="35">
         <v>474</v>
       </c>
@@ -10899,7 +10902,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A190" s="35">
         <v>475</v>
       </c>
@@ -10936,7 +10939,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A191" s="35">
         <v>476</v>
       </c>
@@ -10989,7 +10992,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A192" s="35">
         <v>477</v>
       </c>
@@ -11030,7 +11033,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:23" ht="11.1" customHeight="1" thickBot="1" ns3:dyDescent="0.3">
       <c r="A193" s="35">
         <v>478</v>
       </c>
@@ -11071,7 +11074,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="194" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
       <c r="H194" s="6"/>
@@ -11091,7 +11094,7 @@
       <c r="V194" s="2"/>
       <c r="W194" s="9"/>
     </row>
-    <row r="195" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
       <c r="H195" s="6"/>
@@ -11111,7 +11114,7 @@
       <c r="V195" s="2"/>
       <c r="W195" s="9"/>
     </row>
-    <row r="196" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F196" s="6"/>
       <c r="G196" s="6"/>
       <c r="H196" s="6"/>
@@ -11131,7 +11134,7 @@
       <c r="V196" s="2"/>
       <c r="W196" s="9"/>
     </row>
-    <row r="197" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F197" s="6"/>
       <c r="G197" s="6"/>
       <c r="H197" s="6"/>
@@ -11151,7 +11154,7 @@
       <c r="V197" s="2"/>
       <c r="W197" s="9"/>
     </row>
-    <row r="198" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F198" s="6"/>
       <c r="G198" s="6"/>
       <c r="H198" s="6"/>
@@ -11171,7 +11174,7 @@
       <c r="V198" s="2"/>
       <c r="W198" s="9"/>
     </row>
-    <row r="199" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F199" s="6"/>
       <c r="G199" s="6"/>
       <c r="H199" s="6"/>
@@ -11191,7 +11194,7 @@
       <c r="V199" s="2"/>
       <c r="W199" s="9"/>
     </row>
-    <row r="200" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F200" s="6"/>
       <c r="G200" s="6"/>
       <c r="H200" s="6"/>
@@ -11211,7 +11214,7 @@
       <c r="V200" s="2"/>
       <c r="W200" s="9"/>
     </row>
-    <row r="201" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F201" s="6"/>
       <c r="G201" s="6"/>
       <c r="H201" s="6"/>
@@ -11231,7 +11234,7 @@
       <c r="V201" s="2"/>
       <c r="W201" s="9"/>
     </row>
-    <row r="202" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F202" s="6"/>
       <c r="G202" s="6"/>
       <c r="H202" s="6"/>
@@ -11251,7 +11254,7 @@
       <c r="V202" s="2"/>
       <c r="W202" s="9"/>
     </row>
-    <row r="203" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F203" s="6"/>
       <c r="G203" s="6"/>
       <c r="H203" s="6"/>
@@ -11271,7 +11274,7 @@
       <c r="V203" s="2"/>
       <c r="W203" s="9"/>
     </row>
-    <row r="204" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F204" s="6"/>
       <c r="G204" s="6"/>
       <c r="H204" s="6"/>
@@ -11291,7 +11294,7 @@
       <c r="V204" s="2"/>
       <c r="W204" s="9"/>
     </row>
-    <row r="205" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F205" s="6"/>
       <c r="G205" s="6"/>
       <c r="H205" s="6"/>
@@ -11311,7 +11314,7 @@
       <c r="V205" s="2"/>
       <c r="W205" s="9"/>
     </row>
-    <row r="206" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F206" s="6"/>
       <c r="G206" s="6"/>
       <c r="H206" s="6"/>
@@ -11331,7 +11334,7 @@
       <c r="V206" s="2"/>
       <c r="W206" s="9"/>
     </row>
-    <row r="207" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F207" s="6"/>
       <c r="G207" s="6"/>
       <c r="H207" s="6"/>
@@ -11351,7 +11354,7 @@
       <c r="V207" s="2"/>
       <c r="W207" s="9"/>
     </row>
-    <row r="208" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F208" s="6"/>
       <c r="G208" s="6"/>
       <c r="H208" s="6"/>
@@ -11371,7 +11374,7 @@
       <c r="V208" s="2"/>
       <c r="W208" s="9"/>
     </row>
-    <row r="209" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F209" s="6"/>
       <c r="G209" s="6"/>
       <c r="H209" s="6"/>
@@ -11391,7 +11394,7 @@
       <c r="V209" s="2"/>
       <c r="W209" s="9"/>
     </row>
-    <row r="210" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F210" s="6"/>
       <c r="G210" s="6"/>
       <c r="H210" s="6"/>
@@ -11411,7 +11414,7 @@
       <c r="V210" s="2"/>
       <c r="W210" s="9"/>
     </row>
-    <row r="211" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F211" s="6"/>
       <c r="G211" s="6"/>
       <c r="H211" s="6"/>
@@ -11431,7 +11434,7 @@
       <c r="V211" s="2"/>
       <c r="W211" s="9"/>
     </row>
-    <row r="212" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F212" s="6"/>
       <c r="G212" s="6"/>
       <c r="H212" s="6"/>
@@ -11451,7 +11454,7 @@
       <c r="V212" s="2"/>
       <c r="W212" s="9"/>
     </row>
-    <row r="213" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F213" s="6"/>
       <c r="G213" s="6"/>
       <c r="H213" s="6"/>
@@ -11471,7 +11474,7 @@
       <c r="V213" s="2"/>
       <c r="W213" s="9"/>
     </row>
-    <row r="214" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
       <c r="H214" s="6"/>
@@ -11491,7 +11494,7 @@
       <c r="V214" s="2"/>
       <c r="W214" s="9"/>
     </row>
-    <row r="215" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F215" s="6"/>
       <c r="G215" s="6"/>
       <c r="H215" s="6"/>
@@ -11511,7 +11514,7 @@
       <c r="V215" s="2"/>
       <c r="W215" s="9"/>
     </row>
-    <row r="216" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F216" s="6"/>
       <c r="G216" s="6"/>
       <c r="H216" s="6"/>
@@ -11531,7 +11534,7 @@
       <c r="V216" s="2"/>
       <c r="W216" s="9"/>
     </row>
-    <row r="217" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F217" s="6"/>
       <c r="G217" s="6"/>
       <c r="H217" s="6"/>
@@ -11551,7 +11554,7 @@
       <c r="V217" s="2"/>
       <c r="W217" s="9"/>
     </row>
-    <row r="218" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F218" s="6"/>
       <c r="G218" s="6"/>
       <c r="H218" s="6"/>
@@ -11571,7 +11574,7 @@
       <c r="V218" s="2"/>
       <c r="W218" s="9"/>
     </row>
-    <row r="219" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F219" s="6"/>
       <c r="G219" s="6"/>
       <c r="H219" s="6"/>
@@ -11591,7 +11594,7 @@
       <c r="V219" s="2"/>
       <c r="W219" s="9"/>
     </row>
-    <row r="220" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F220" s="6"/>
       <c r="G220" s="6"/>
       <c r="H220" s="6"/>
@@ -11611,7 +11614,7 @@
       <c r="V220" s="2"/>
       <c r="W220" s="9"/>
     </row>
-    <row r="221" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F221" s="6"/>
       <c r="G221" s="6"/>
       <c r="H221" s="6"/>
@@ -11631,7 +11634,7 @@
       <c r="V221" s="2"/>
       <c r="W221" s="9"/>
     </row>
-    <row r="222" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F222" s="6"/>
       <c r="G222" s="6"/>
       <c r="H222" s="6"/>
@@ -11651,7 +11654,7 @@
       <c r="V222" s="2"/>
       <c r="W222" s="9"/>
     </row>
-    <row r="223" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F223" s="6"/>
       <c r="G223" s="6"/>
       <c r="H223" s="6"/>
@@ -11671,7 +11674,7 @@
       <c r="V223" s="2"/>
       <c r="W223" s="9"/>
     </row>
-    <row r="224" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F224" s="6"/>
       <c r="G224" s="6"/>
       <c r="H224" s="6"/>
@@ -11691,7 +11694,7 @@
       <c r="V224" s="2"/>
       <c r="W224" s="9"/>
     </row>
-    <row r="225" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F225" s="6"/>
       <c r="G225" s="6"/>
       <c r="H225" s="6"/>
@@ -11711,7 +11714,7 @@
       <c r="V225" s="2"/>
       <c r="W225" s="9"/>
     </row>
-    <row r="226" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F226" s="6"/>
       <c r="G226" s="6"/>
       <c r="H226" s="6"/>
@@ -11731,7 +11734,7 @@
       <c r="V226" s="2"/>
       <c r="W226" s="9"/>
     </row>
-    <row r="227" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F227" s="6"/>
       <c r="G227" s="6"/>
       <c r="H227" s="6"/>
@@ -11751,7 +11754,7 @@
       <c r="V227" s="2"/>
       <c r="W227" s="9"/>
     </row>
-    <row r="228" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F228" s="6"/>
       <c r="G228" s="6"/>
       <c r="H228" s="6"/>
@@ -11771,7 +11774,7 @@
       <c r="V228" s="2"/>
       <c r="W228" s="9"/>
     </row>
-    <row r="229" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F229" s="6"/>
       <c r="G229" s="6"/>
       <c r="H229" s="6"/>
@@ -11791,7 +11794,7 @@
       <c r="V229" s="2"/>
       <c r="W229" s="9"/>
     </row>
-    <row r="230" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F230" s="6"/>
       <c r="G230" s="6"/>
       <c r="H230" s="6"/>
@@ -11811,7 +11814,7 @@
       <c r="V230" s="2"/>
       <c r="W230" s="9"/>
     </row>
-    <row r="231" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F231" s="6"/>
       <c r="G231" s="6"/>
       <c r="H231" s="6"/>
@@ -11831,7 +11834,7 @@
       <c r="V231" s="2"/>
       <c r="W231" s="9"/>
     </row>
-    <row r="232" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F232" s="6"/>
       <c r="G232" s="6"/>
       <c r="H232" s="6"/>
@@ -11851,7 +11854,7 @@
       <c r="V232" s="2"/>
       <c r="W232" s="9"/>
     </row>
-    <row r="233" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F233" s="6"/>
       <c r="G233" s="6"/>
       <c r="H233" s="6"/>
@@ -11871,7 +11874,7 @@
       <c r="V233" s="2"/>
       <c r="W233" s="9"/>
     </row>
-    <row r="234" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F234" s="6"/>
       <c r="G234" s="6"/>
       <c r="H234" s="6"/>
@@ -11891,7 +11894,7 @@
       <c r="V234" s="2"/>
       <c r="W234" s="9"/>
     </row>
-    <row r="235" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F235" s="6"/>
       <c r="G235" s="6"/>
       <c r="H235" s="6"/>
@@ -11911,7 +11914,7 @@
       <c r="V235" s="2"/>
       <c r="W235" s="9"/>
     </row>
-    <row r="236" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F236" s="6"/>
       <c r="G236" s="6"/>
       <c r="H236" s="6"/>
@@ -11931,7 +11934,7 @@
       <c r="V236" s="2"/>
       <c r="W236" s="9"/>
     </row>
-    <row r="237" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F237" s="6"/>
       <c r="G237" s="6"/>
       <c r="H237" s="6"/>
@@ -11951,7 +11954,7 @@
       <c r="V237" s="2"/>
       <c r="W237" s="9"/>
     </row>
-    <row r="238" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F238" s="6"/>
       <c r="G238" s="6"/>
       <c r="H238" s="6"/>
@@ -11971,7 +11974,7 @@
       <c r="V238" s="2"/>
       <c r="W238" s="9"/>
     </row>
-    <row r="239" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F239" s="6"/>
       <c r="G239" s="6"/>
       <c r="H239" s="6"/>
@@ -11991,7 +11994,7 @@
       <c r="V239" s="2"/>
       <c r="W239" s="9"/>
     </row>
-    <row r="240" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F240" s="6"/>
       <c r="G240" s="6"/>
       <c r="H240" s="6"/>
@@ -12011,7 +12014,7 @@
       <c r="V240" s="2"/>
       <c r="W240" s="9"/>
     </row>
-    <row r="241" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F241" s="6"/>
       <c r="G241" s="6"/>
       <c r="H241" s="6"/>
@@ -12031,7 +12034,7 @@
       <c r="V241" s="2"/>
       <c r="W241" s="9"/>
     </row>
-    <row r="242" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F242" s="6"/>
       <c r="G242" s="6"/>
       <c r="H242" s="6"/>
@@ -12051,7 +12054,7 @@
       <c r="V242" s="2"/>
       <c r="W242" s="9"/>
     </row>
-    <row r="243" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F243" s="6"/>
       <c r="G243" s="6"/>
       <c r="H243" s="6"/>
@@ -12071,7 +12074,7 @@
       <c r="V243" s="2"/>
       <c r="W243" s="9"/>
     </row>
-    <row r="244" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F244" s="6"/>
       <c r="G244" s="6"/>
       <c r="H244" s="6"/>
@@ -12091,7 +12094,7 @@
       <c r="V244" s="2"/>
       <c r="W244" s="9"/>
     </row>
-    <row r="245" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F245" s="6"/>
       <c r="G245" s="6"/>
       <c r="H245" s="6"/>
@@ -12111,7 +12114,7 @@
       <c r="V245" s="2"/>
       <c r="W245" s="9"/>
     </row>
-    <row r="246" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F246" s="6"/>
       <c r="G246" s="6"/>
       <c r="H246" s="6"/>
@@ -12131,7 +12134,7 @@
       <c r="V246" s="2"/>
       <c r="W246" s="9"/>
     </row>
-    <row r="247" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F247" s="6"/>
       <c r="G247" s="6"/>
       <c r="H247" s="6"/>
@@ -12151,7 +12154,7 @@
       <c r="V247" s="2"/>
       <c r="W247" s="9"/>
     </row>
-    <row r="248" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F248" s="6"/>
       <c r="G248" s="6"/>
       <c r="H248" s="6"/>
@@ -12171,7 +12174,7 @@
       <c r="V248" s="2"/>
       <c r="W248" s="9"/>
     </row>
-    <row r="249" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F249" s="6"/>
       <c r="G249" s="6"/>
       <c r="H249" s="6"/>
@@ -12191,7 +12194,7 @@
       <c r="V249" s="2"/>
       <c r="W249" s="9"/>
     </row>
-    <row r="250" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F250" s="6"/>
       <c r="G250" s="6"/>
       <c r="H250" s="6"/>
@@ -12211,7 +12214,7 @@
       <c r="V250" s="2"/>
       <c r="W250" s="9"/>
     </row>
-    <row r="251" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F251" s="6"/>
       <c r="G251" s="6"/>
       <c r="H251" s="6"/>
@@ -12231,7 +12234,7 @@
       <c r="V251" s="2"/>
       <c r="W251" s="9"/>
     </row>
-    <row r="252" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F252" s="6"/>
       <c r="G252" s="6"/>
       <c r="H252" s="6"/>
@@ -12251,7 +12254,7 @@
       <c r="V252" s="2"/>
       <c r="W252" s="9"/>
     </row>
-    <row r="253" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F253" s="6"/>
       <c r="G253" s="6"/>
       <c r="H253" s="6"/>
@@ -12271,7 +12274,7 @@
       <c r="V253" s="2"/>
       <c r="W253" s="9"/>
     </row>
-    <row r="254" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F254" s="6"/>
       <c r="G254" s="6"/>
       <c r="H254" s="6"/>
@@ -12291,7 +12294,7 @@
       <c r="V254" s="2"/>
       <c r="W254" s="9"/>
     </row>
-    <row r="255" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F255" s="6"/>
       <c r="G255" s="6"/>
       <c r="H255" s="6"/>
@@ -12311,7 +12314,7 @@
       <c r="V255" s="2"/>
       <c r="W255" s="9"/>
     </row>
-    <row r="256" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F256" s="6"/>
       <c r="G256" s="6"/>
       <c r="H256" s="6"/>
@@ -12331,7 +12334,7 @@
       <c r="V256" s="2"/>
       <c r="W256" s="9"/>
     </row>
-    <row r="257" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F257" s="6"/>
       <c r="G257" s="6"/>
       <c r="H257" s="6"/>
@@ -12351,7 +12354,7 @@
       <c r="V257" s="2"/>
       <c r="W257" s="9"/>
     </row>
-    <row r="258" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F258" s="6"/>
       <c r="G258" s="6"/>
       <c r="H258" s="6"/>
@@ -12371,7 +12374,7 @@
       <c r="V258" s="2"/>
       <c r="W258" s="9"/>
     </row>
-    <row r="259" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F259" s="6"/>
       <c r="G259" s="6"/>
       <c r="H259" s="6"/>
@@ -12391,7 +12394,7 @@
       <c r="V259" s="2"/>
       <c r="W259" s="9"/>
     </row>
-    <row r="260" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F260" s="6"/>
       <c r="G260" s="6"/>
       <c r="H260" s="6"/>
@@ -12411,7 +12414,7 @@
       <c r="V260" s="2"/>
       <c r="W260" s="9"/>
     </row>
-    <row r="261" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F261" s="6"/>
       <c r="G261" s="6"/>
       <c r="H261" s="6"/>
@@ -12431,7 +12434,7 @@
       <c r="V261" s="2"/>
       <c r="W261" s="9"/>
     </row>
-    <row r="262" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F262" s="6"/>
       <c r="G262" s="6"/>
       <c r="H262" s="6"/>
@@ -12451,7 +12454,7 @@
       <c r="V262" s="2"/>
       <c r="W262" s="9"/>
     </row>
-    <row r="263" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F263" s="6"/>
       <c r="G263" s="6"/>
       <c r="H263" s="6"/>
@@ -12471,7 +12474,7 @@
       <c r="V263" s="2"/>
       <c r="W263" s="9"/>
     </row>
-    <row r="264" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F264" s="6"/>
       <c r="G264" s="6"/>
       <c r="H264" s="6"/>
@@ -12491,7 +12494,7 @@
       <c r="V264" s="2"/>
       <c r="W264" s="9"/>
     </row>
-    <row r="265" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F265" s="6"/>
       <c r="G265" s="6"/>
       <c r="H265" s="6"/>
@@ -12511,7 +12514,7 @@
       <c r="V265" s="2"/>
       <c r="W265" s="9"/>
     </row>
-    <row r="266" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F266" s="6"/>
       <c r="G266" s="6"/>
       <c r="H266" s="6"/>
@@ -12531,7 +12534,7 @@
       <c r="V266" s="2"/>
       <c r="W266" s="9"/>
     </row>
-    <row r="267" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F267" s="6"/>
       <c r="G267" s="6"/>
       <c r="H267" s="6"/>
@@ -12551,7 +12554,7 @@
       <c r="V267" s="2"/>
       <c r="W267" s="9"/>
     </row>
-    <row r="268" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F268" s="6"/>
       <c r="G268" s="6"/>
       <c r="H268" s="6"/>
@@ -12571,7 +12574,7 @@
       <c r="V268" s="2"/>
       <c r="W268" s="9"/>
     </row>
-    <row r="269" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F269" s="6"/>
       <c r="G269" s="6"/>
       <c r="H269" s="6"/>
@@ -12591,7 +12594,7 @@
       <c r="V269" s="2"/>
       <c r="W269" s="9"/>
     </row>
-    <row r="270" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F270" s="6"/>
       <c r="G270" s="6"/>
       <c r="H270" s="6"/>
@@ -12611,7 +12614,7 @@
       <c r="V270" s="2"/>
       <c r="W270" s="9"/>
     </row>
-    <row r="271" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F271" s="6"/>
       <c r="G271" s="6"/>
       <c r="H271" s="6"/>
@@ -12631,7 +12634,7 @@
       <c r="V271" s="2"/>
       <c r="W271" s="9"/>
     </row>
-    <row r="272" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F272" s="6"/>
       <c r="G272" s="6"/>
       <c r="H272" s="6"/>
@@ -12651,7 +12654,7 @@
       <c r="V272" s="2"/>
       <c r="W272" s="9"/>
     </row>
-    <row r="273" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F273" s="6"/>
       <c r="G273" s="6"/>
       <c r="H273" s="6"/>
@@ -12671,7 +12674,7 @@
       <c r="V273" s="2"/>
       <c r="W273" s="9"/>
     </row>
-    <row r="274" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F274" s="6"/>
       <c r="G274" s="6"/>
       <c r="H274" s="6"/>
@@ -12691,7 +12694,7 @@
       <c r="V274" s="2"/>
       <c r="W274" s="9"/>
     </row>
-    <row r="275" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F275" s="6"/>
       <c r="G275" s="6"/>
       <c r="H275" s="6"/>
@@ -12711,7 +12714,7 @@
       <c r="V275" s="2"/>
       <c r="W275" s="9"/>
     </row>
-    <row r="276" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F276" s="6"/>
       <c r="G276" s="6"/>
       <c r="H276" s="6"/>
@@ -12731,7 +12734,7 @@
       <c r="V276" s="2"/>
       <c r="W276" s="9"/>
     </row>
-    <row r="277" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F277" s="6"/>
       <c r="G277" s="6"/>
       <c r="H277" s="6"/>
@@ -12751,7 +12754,7 @@
       <c r="V277" s="2"/>
       <c r="W277" s="9"/>
     </row>
-    <row r="278" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F278" s="6"/>
       <c r="G278" s="6"/>
       <c r="H278" s="6"/>
@@ -12771,7 +12774,7 @@
       <c r="V278" s="2"/>
       <c r="W278" s="9"/>
     </row>
-    <row r="279" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F279" s="6"/>
       <c r="G279" s="6"/>
       <c r="H279" s="6"/>
@@ -12791,7 +12794,7 @@
       <c r="V279" s="2"/>
       <c r="W279" s="9"/>
     </row>
-    <row r="280" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F280" s="6"/>
       <c r="G280" s="6"/>
       <c r="H280" s="6"/>
@@ -12811,7 +12814,7 @@
       <c r="V280" s="2"/>
       <c r="W280" s="9"/>
     </row>
-    <row r="281" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F281" s="6"/>
       <c r="G281" s="6"/>
       <c r="H281" s="6"/>
@@ -12831,7 +12834,7 @@
       <c r="V281" s="2"/>
       <c r="W281" s="9"/>
     </row>
-    <row r="282" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F282" s="6"/>
       <c r="G282" s="6"/>
       <c r="H282" s="6"/>
@@ -12851,7 +12854,7 @@
       <c r="V282" s="2"/>
       <c r="W282" s="9"/>
     </row>
-    <row r="283" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F283" s="6"/>
       <c r="G283" s="6"/>
       <c r="H283" s="6"/>
@@ -12871,7 +12874,7 @@
       <c r="V283" s="2"/>
       <c r="W283" s="9"/>
     </row>
-    <row r="284" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F284" s="6"/>
       <c r="G284" s="6"/>
       <c r="H284" s="6"/>
@@ -12891,7 +12894,7 @@
       <c r="V284" s="2"/>
       <c r="W284" s="9"/>
     </row>
-    <row r="285" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F285" s="6"/>
       <c r="G285" s="6"/>
       <c r="H285" s="6"/>
@@ -12911,7 +12914,7 @@
       <c r="V285" s="2"/>
       <c r="W285" s="9"/>
     </row>
-    <row r="286" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F286" s="6"/>
       <c r="G286" s="6"/>
       <c r="H286" s="6"/>
@@ -12931,7 +12934,7 @@
       <c r="V286" s="2"/>
       <c r="W286" s="9"/>
     </row>
-    <row r="287" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F287" s="6"/>
       <c r="G287" s="6"/>
       <c r="H287" s="6"/>
@@ -12951,7 +12954,7 @@
       <c r="V287" s="2"/>
       <c r="W287" s="9"/>
     </row>
-    <row r="288" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F288" s="6"/>
       <c r="G288" s="6"/>
       <c r="H288" s="6"/>
@@ -12971,7 +12974,7 @@
       <c r="V288" s="2"/>
       <c r="W288" s="9"/>
     </row>
-    <row r="289" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F289" s="6"/>
       <c r="G289" s="6"/>
       <c r="H289" s="6"/>
@@ -12991,7 +12994,7 @@
       <c r="V289" s="2"/>
       <c r="W289" s="9"/>
     </row>
-    <row r="290" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F290" s="6"/>
       <c r="G290" s="6"/>
       <c r="H290" s="6"/>
@@ -13011,7 +13014,7 @@
       <c r="V290" s="2"/>
       <c r="W290" s="9"/>
     </row>
-    <row r="291" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F291" s="6"/>
       <c r="G291" s="6"/>
       <c r="H291" s="6"/>
@@ -13031,7 +13034,7 @@
       <c r="V291" s="2"/>
       <c r="W291" s="9"/>
     </row>
-    <row r="292" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F292" s="6"/>
       <c r="G292" s="6"/>
       <c r="H292" s="6"/>
@@ -13051,7 +13054,7 @@
       <c r="V292" s="2"/>
       <c r="W292" s="9"/>
     </row>
-    <row r="293" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F293" s="6"/>
       <c r="G293" s="6"/>
       <c r="H293" s="6"/>
@@ -13071,7 +13074,7 @@
       <c r="V293" s="2"/>
       <c r="W293" s="9"/>
     </row>
-    <row r="294" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F294" s="6"/>
       <c r="G294" s="6"/>
       <c r="H294" s="6"/>
@@ -13091,7 +13094,7 @@
       <c r="V294" s="2"/>
       <c r="W294" s="9"/>
     </row>
-    <row r="295" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F295" s="6"/>
       <c r="G295" s="6"/>
       <c r="H295" s="6"/>
@@ -13111,7 +13114,7 @@
       <c r="V295" s="2"/>
       <c r="W295" s="9"/>
     </row>
-    <row r="296" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F296" s="6"/>
       <c r="G296" s="6"/>
       <c r="H296" s="6"/>
@@ -13131,7 +13134,7 @@
       <c r="V296" s="2"/>
       <c r="W296" s="9"/>
     </row>
-    <row r="297" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F297" s="6"/>
       <c r="G297" s="6"/>
       <c r="H297" s="6"/>
@@ -13151,7 +13154,7 @@
       <c r="V297" s="2"/>
       <c r="W297" s="9"/>
     </row>
-    <row r="298" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F298" s="6"/>
       <c r="G298" s="6"/>
       <c r="H298" s="6"/>
@@ -13171,7 +13174,7 @@
       <c r="V298" s="2"/>
       <c r="W298" s="9"/>
     </row>
-    <row r="299" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F299" s="6"/>
       <c r="G299" s="6"/>
       <c r="H299" s="6"/>
@@ -13191,7 +13194,7 @@
       <c r="V299" s="2"/>
       <c r="W299" s="9"/>
     </row>
-    <row r="300" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F300" s="6"/>
       <c r="G300" s="6"/>
       <c r="H300" s="6"/>
@@ -13211,7 +13214,7 @@
       <c r="V300" s="2"/>
       <c r="W300" s="9"/>
     </row>
-    <row r="301" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F301" s="6"/>
       <c r="G301" s="6"/>
       <c r="H301" s="6"/>
@@ -13231,7 +13234,7 @@
       <c r="V301" s="2"/>
       <c r="W301" s="9"/>
     </row>
-    <row r="302" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F302" s="6"/>
       <c r="G302" s="6"/>
       <c r="H302" s="6"/>
@@ -13251,7 +13254,7 @@
       <c r="V302" s="2"/>
       <c r="W302" s="9"/>
     </row>
-    <row r="303" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F303" s="6"/>
       <c r="G303" s="6"/>
       <c r="H303" s="6"/>
@@ -13271,7 +13274,7 @@
       <c r="V303" s="2"/>
       <c r="W303" s="9"/>
     </row>
-    <row r="304" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F304" s="6"/>
       <c r="G304" s="6"/>
       <c r="H304" s="6"/>
@@ -13291,7 +13294,7 @@
       <c r="V304" s="2"/>
       <c r="W304" s="9"/>
     </row>
-    <row r="305" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F305" s="6"/>
       <c r="G305" s="6"/>
       <c r="H305" s="6"/>
@@ -13311,7 +13314,7 @@
       <c r="V305" s="2"/>
       <c r="W305" s="9"/>
     </row>
-    <row r="306" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F306" s="6"/>
       <c r="G306" s="6"/>
       <c r="H306" s="6"/>
@@ -13331,7 +13334,7 @@
       <c r="V306" s="2"/>
       <c r="W306" s="9"/>
     </row>
-    <row r="307" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F307" s="6"/>
       <c r="G307" s="6"/>
       <c r="H307" s="6"/>
@@ -13351,7 +13354,7 @@
       <c r="V307" s="2"/>
       <c r="W307" s="9"/>
     </row>
-    <row r="308" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F308" s="6"/>
       <c r="G308" s="6"/>
       <c r="H308" s="6"/>
@@ -13371,7 +13374,7 @@
       <c r="V308" s="2"/>
       <c r="W308" s="9"/>
     </row>
-    <row r="309" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F309" s="6"/>
       <c r="G309" s="6"/>
       <c r="H309" s="6"/>
@@ -13391,7 +13394,7 @@
       <c r="V309" s="2"/>
       <c r="W309" s="9"/>
     </row>
-    <row r="310" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F310" s="6"/>
       <c r="G310" s="6"/>
       <c r="H310" s="6"/>
@@ -13411,7 +13414,7 @@
       <c r="V310" s="2"/>
       <c r="W310" s="9"/>
     </row>
-    <row r="311" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F311" s="6"/>
       <c r="G311" s="6"/>
       <c r="H311" s="6"/>
@@ -13431,7 +13434,7 @@
       <c r="V311" s="2"/>
       <c r="W311" s="9"/>
     </row>
-    <row r="312" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F312" s="6"/>
       <c r="G312" s="6"/>
       <c r="H312" s="6"/>
@@ -13451,7 +13454,7 @@
       <c r="V312" s="2"/>
       <c r="W312" s="9"/>
     </row>
-    <row r="313" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F313" s="6"/>
       <c r="G313" s="6"/>
       <c r="H313" s="6"/>
@@ -13471,7 +13474,7 @@
       <c r="V313" s="2"/>
       <c r="W313" s="9"/>
     </row>
-    <row r="314" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F314" s="6"/>
       <c r="G314" s="6"/>
       <c r="H314" s="6"/>
@@ -13491,7 +13494,7 @@
       <c r="V314" s="2"/>
       <c r="W314" s="9"/>
     </row>
-    <row r="315" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F315" s="6"/>
       <c r="G315" s="6"/>
       <c r="H315" s="6"/>
@@ -13511,7 +13514,7 @@
       <c r="V315" s="2"/>
       <c r="W315" s="9"/>
     </row>
-    <row r="316" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F316" s="6"/>
       <c r="G316" s="6"/>
       <c r="H316" s="6"/>
@@ -13531,7 +13534,7 @@
       <c r="V316" s="2"/>
       <c r="W316" s="9"/>
     </row>
-    <row r="317" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F317" s="6"/>
       <c r="G317" s="6"/>
       <c r="H317" s="6"/>
@@ -13551,7 +13554,7 @@
       <c r="V317" s="2"/>
       <c r="W317" s="9"/>
     </row>
-    <row r="318" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F318" s="6"/>
       <c r="G318" s="6"/>
       <c r="H318" s="6"/>
@@ -13571,7 +13574,7 @@
       <c r="V318" s="2"/>
       <c r="W318" s="9"/>
     </row>
-    <row r="319" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F319" s="6"/>
       <c r="G319" s="6"/>
       <c r="H319" s="6"/>
@@ -13591,7 +13594,7 @@
       <c r="V319" s="2"/>
       <c r="W319" s="9"/>
     </row>
-    <row r="320" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F320" s="6"/>
       <c r="G320" s="6"/>
       <c r="H320" s="6"/>
@@ -13611,7 +13614,7 @@
       <c r="V320" s="2"/>
       <c r="W320" s="9"/>
     </row>
-    <row r="321" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F321" s="6"/>
       <c r="G321" s="6"/>
       <c r="H321" s="6"/>
@@ -13631,7 +13634,7 @@
       <c r="V321" s="2"/>
       <c r="W321" s="9"/>
     </row>
-    <row r="322" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F322" s="6"/>
       <c r="G322" s="6"/>
       <c r="H322" s="6"/>
@@ -13651,7 +13654,7 @@
       <c r="V322" s="2"/>
       <c r="W322" s="9"/>
     </row>
-    <row r="323" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F323" s="6"/>
       <c r="G323" s="6"/>
       <c r="H323" s="6"/>
@@ -13671,7 +13674,7 @@
       <c r="V323" s="2"/>
       <c r="W323" s="9"/>
     </row>
-    <row r="324" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F324" s="6"/>
       <c r="G324" s="6"/>
       <c r="H324" s="6"/>
@@ -13691,7 +13694,7 @@
       <c r="V324" s="2"/>
       <c r="W324" s="9"/>
     </row>
-    <row r="325" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F325" s="6"/>
       <c r="G325" s="6"/>
       <c r="H325" s="6"/>
@@ -13711,7 +13714,7 @@
       <c r="V325" s="2"/>
       <c r="W325" s="9"/>
     </row>
-    <row r="326" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F326" s="6"/>
       <c r="G326" s="6"/>
       <c r="H326" s="6"/>
@@ -13731,7 +13734,7 @@
       <c r="V326" s="2"/>
       <c r="W326" s="9"/>
     </row>
-    <row r="327" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F327" s="6"/>
       <c r="G327" s="6"/>
       <c r="H327" s="6"/>
@@ -13751,7 +13754,7 @@
       <c r="V327" s="2"/>
       <c r="W327" s="9"/>
     </row>
-    <row r="328" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="F328" s="6"/>
       <c r="G328" s="6"/>
       <c r="H328" s="6"/>
@@ -13771,1270 +13774,1270 @@
       <c r="V328" s="2"/>
       <c r="W328" s="9"/>
     </row>
-    <row r="329" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W329" s="7"/>
     </row>
-    <row r="330" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W330" s="7"/>
     </row>
-    <row r="331" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W331" s="7"/>
     </row>
-    <row r="332" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W332" s="7"/>
     </row>
-    <row r="333" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W333" s="7"/>
     </row>
-    <row r="334" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W334" s="7"/>
     </row>
-    <row r="335" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W335" s="7"/>
     </row>
-    <row r="336" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="6:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W336" s="7"/>
     </row>
-    <row r="337" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W337" s="7"/>
     </row>
-    <row r="338" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W338" s="7"/>
     </row>
-    <row r="339" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W339" s="7"/>
     </row>
-    <row r="340" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W340" s="7"/>
     </row>
-    <row r="341" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W341" s="7"/>
     </row>
-    <row r="342" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W342" s="7"/>
     </row>
-    <row r="343" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W343" s="7"/>
     </row>
-    <row r="344" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W344" s="7"/>
     </row>
-    <row r="345" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W345" s="7"/>
     </row>
-    <row r="346" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W346" s="7"/>
     </row>
-    <row r="347" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W347" s="7"/>
     </row>
-    <row r="348" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W348" s="7"/>
     </row>
-    <row r="349" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W349" s="7"/>
     </row>
-    <row r="350" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W350" s="7"/>
     </row>
-    <row r="351" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W351" s="7"/>
     </row>
-    <row r="352" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W352" s="7"/>
     </row>
-    <row r="353" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W353" s="7"/>
     </row>
-    <row r="354" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W354" s="7"/>
     </row>
-    <row r="355" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W355" s="7"/>
     </row>
-    <row r="356" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W356" s="7"/>
     </row>
-    <row r="357" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W357" s="7"/>
     </row>
-    <row r="358" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W358" s="7"/>
     </row>
-    <row r="359" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W359" s="7"/>
     </row>
-    <row r="360" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W360" s="7"/>
     </row>
-    <row r="361" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W361" s="7"/>
     </row>
-    <row r="362" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W362" s="7"/>
     </row>
-    <row r="363" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W363" s="7"/>
     </row>
-    <row r="364" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W364" s="7"/>
     </row>
-    <row r="365" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W365" s="7"/>
     </row>
-    <row r="366" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W366" s="7"/>
     </row>
-    <row r="367" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W367" s="7"/>
     </row>
-    <row r="368" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W368" s="7"/>
     </row>
-    <row r="369" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W369" s="7"/>
     </row>
-    <row r="370" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W370" s="7"/>
     </row>
-    <row r="371" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W371" s="7"/>
     </row>
-    <row r="372" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W372" s="7"/>
     </row>
-    <row r="373" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W373" s="7"/>
     </row>
-    <row r="374" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W374" s="7"/>
     </row>
-    <row r="375" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W375" s="7"/>
     </row>
-    <row r="376" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W376" s="7"/>
     </row>
-    <row r="377" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W377" s="7"/>
     </row>
-    <row r="378" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W378" s="7"/>
     </row>
-    <row r="379" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W379" s="7"/>
     </row>
-    <row r="380" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W380" s="7"/>
     </row>
-    <row r="381" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W381" s="7"/>
     </row>
-    <row r="382" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W382" s="7"/>
     </row>
-    <row r="383" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W383" s="7"/>
     </row>
-    <row r="384" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W384" s="7"/>
     </row>
-    <row r="385" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W385" s="7"/>
     </row>
-    <row r="386" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W386" s="7"/>
     </row>
-    <row r="387" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W387" s="7"/>
     </row>
-    <row r="388" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W388" s="7"/>
     </row>
-    <row r="389" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W389" s="7"/>
     </row>
-    <row r="390" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W390" s="7"/>
     </row>
-    <row r="391" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W391" s="7"/>
     </row>
-    <row r="392" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W392" s="7"/>
     </row>
-    <row r="393" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W393" s="7"/>
     </row>
-    <row r="394" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W394" s="7"/>
     </row>
-    <row r="395" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W395" s="7"/>
     </row>
-    <row r="396" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W396" s="7"/>
     </row>
-    <row r="397" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W397" s="7"/>
     </row>
-    <row r="398" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W398" s="7"/>
     </row>
-    <row r="399" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W399" s="7"/>
     </row>
-    <row r="400" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W400" s="7"/>
     </row>
-    <row r="401" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W401" s="7"/>
     </row>
-    <row r="402" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W402" s="7"/>
     </row>
-    <row r="403" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W403" s="7"/>
     </row>
-    <row r="404" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W404" s="7"/>
     </row>
-    <row r="405" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W405" s="7"/>
     </row>
-    <row r="406" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W406" s="7"/>
     </row>
-    <row r="407" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W407" s="7"/>
     </row>
-    <row r="408" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W408" s="7"/>
     </row>
-    <row r="409" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W409" s="7"/>
     </row>
-    <row r="410" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W410" s="7"/>
     </row>
-    <row r="411" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W411" s="7"/>
     </row>
-    <row r="412" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W412" s="7"/>
     </row>
-    <row r="413" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W413" s="7"/>
     </row>
-    <row r="414" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W414" s="7"/>
     </row>
-    <row r="415" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W415" s="7"/>
     </row>
-    <row r="416" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W416" s="7"/>
     </row>
-    <row r="417" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W417" s="7"/>
     </row>
-    <row r="418" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W418" s="7"/>
     </row>
-    <row r="419" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W419" s="7"/>
     </row>
-    <row r="420" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W420" s="7"/>
     </row>
-    <row r="421" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W421" s="7"/>
     </row>
-    <row r="422" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W422" s="7"/>
     </row>
-    <row r="423" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W423" s="7"/>
     </row>
-    <row r="424" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W424" s="7"/>
     </row>
-    <row r="425" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W425" s="7"/>
     </row>
-    <row r="426" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W426" s="7"/>
     </row>
-    <row r="427" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W427" s="7"/>
     </row>
-    <row r="428" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W428" s="7"/>
     </row>
-    <row r="429" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W429" s="7"/>
     </row>
-    <row r="430" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W430" s="7"/>
     </row>
-    <row r="431" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="431" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W431" s="7"/>
     </row>
-    <row r="432" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W432" s="7"/>
     </row>
-    <row r="433" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W433" s="7"/>
     </row>
-    <row r="434" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="434" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W434" s="7"/>
     </row>
-    <row r="435" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W435" s="7"/>
     </row>
-    <row r="436" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W436" s="7"/>
     </row>
-    <row r="437" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="437" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W437" s="7"/>
     </row>
-    <row r="438" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W438" s="7"/>
     </row>
-    <row r="439" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W439" s="7"/>
     </row>
-    <row r="440" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W440" s="7"/>
     </row>
-    <row r="441" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W441" s="7"/>
     </row>
-    <row r="442" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W442" s="7"/>
     </row>
-    <row r="443" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W443" s="7"/>
     </row>
-    <row r="444" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W444" s="7"/>
     </row>
-    <row r="445" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W445" s="7"/>
     </row>
-    <row r="446" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W446" s="7"/>
     </row>
-    <row r="447" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W447" s="7"/>
     </row>
-    <row r="448" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W448" s="7"/>
     </row>
-    <row r="449" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W449" s="7"/>
     </row>
-    <row r="450" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W450" s="7"/>
     </row>
-    <row r="451" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W451" s="7"/>
     </row>
-    <row r="452" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W452" s="7"/>
     </row>
-    <row r="453" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W453" s="7"/>
     </row>
-    <row r="454" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W454" s="7"/>
     </row>
-    <row r="455" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W455" s="7"/>
     </row>
-    <row r="456" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W456" s="7"/>
     </row>
-    <row r="457" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W457" s="7"/>
     </row>
-    <row r="458" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W458" s="7"/>
     </row>
-    <row r="459" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W459" s="7"/>
     </row>
-    <row r="460" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W460" s="7"/>
     </row>
-    <row r="461" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W461" s="7"/>
     </row>
-    <row r="462" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W462" s="7"/>
     </row>
-    <row r="463" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W463" s="7"/>
     </row>
-    <row r="464" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W464" s="7"/>
     </row>
-    <row r="465" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W465" s="7"/>
     </row>
-    <row r="466" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W466" s="7"/>
     </row>
-    <row r="467" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W467" s="7"/>
     </row>
-    <row r="468" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W468" s="7"/>
     </row>
-    <row r="469" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="469" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W469" s="7"/>
     </row>
-    <row r="470" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W470" s="7"/>
     </row>
-    <row r="471" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W471" s="7"/>
     </row>
-    <row r="472" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W472" s="7"/>
     </row>
-    <row r="473" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W473" s="7"/>
     </row>
-    <row r="474" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W474" s="7"/>
     </row>
-    <row r="475" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W475" s="7"/>
     </row>
-    <row r="476" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W476" s="7"/>
     </row>
-    <row r="477" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W477" s="7"/>
     </row>
-    <row r="478" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W478" s="7"/>
     </row>
-    <row r="479" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W479" s="7"/>
     </row>
-    <row r="480" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W480" s="7"/>
     </row>
-    <row r="481" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="481" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W481" s="7"/>
     </row>
-    <row r="482" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="482" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W482" s="7"/>
     </row>
-    <row r="483" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="483" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W483" s="7"/>
     </row>
-    <row r="484" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="484" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W484" s="7"/>
     </row>
-    <row r="485" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="485" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W485" s="7"/>
     </row>
-    <row r="486" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="486" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W486" s="7"/>
     </row>
-    <row r="487" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="487" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W487" s="7"/>
     </row>
-    <row r="488" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="488" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W488" s="7"/>
     </row>
-    <row r="489" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="489" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W489" s="7"/>
     </row>
-    <row r="490" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="490" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W490" s="7"/>
     </row>
-    <row r="491" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="491" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W491" s="7"/>
     </row>
-    <row r="492" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="492" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W492" s="7"/>
     </row>
-    <row r="493" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="493" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W493" s="7"/>
     </row>
-    <row r="494" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="494" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W494" s="7"/>
     </row>
-    <row r="495" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="495" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W495" s="7"/>
     </row>
-    <row r="496" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="496" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W496" s="7"/>
     </row>
-    <row r="497" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="497" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W497" s="7"/>
     </row>
-    <row r="498" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="498" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W498" s="7"/>
     </row>
-    <row r="499" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="499" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W499" s="7"/>
     </row>
-    <row r="500" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="500" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W500" s="7"/>
     </row>
-    <row r="501" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="501" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W501" s="7"/>
     </row>
-    <row r="502" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="502" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W502" s="7"/>
     </row>
-    <row r="503" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="503" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W503" s="7"/>
     </row>
-    <row r="504" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="504" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W504" s="7"/>
     </row>
-    <row r="505" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="505" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W505" s="7"/>
     </row>
-    <row r="506" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="506" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W506" s="7"/>
     </row>
-    <row r="507" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="507" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W507" s="7"/>
     </row>
-    <row r="508" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="508" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W508" s="7"/>
     </row>
-    <row r="509" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="509" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W509" s="7"/>
     </row>
-    <row r="510" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="510" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W510" s="7"/>
     </row>
-    <row r="511" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="511" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W511" s="7"/>
     </row>
-    <row r="512" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="512" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W512" s="7"/>
     </row>
-    <row r="513" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="513" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W513" s="7"/>
     </row>
-    <row r="514" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="514" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W514" s="7"/>
     </row>
-    <row r="515" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="515" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W515" s="7"/>
     </row>
-    <row r="516" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="516" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W516" s="7"/>
     </row>
-    <row r="517" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="517" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W517" s="7"/>
     </row>
-    <row r="518" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="518" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W518" s="7"/>
     </row>
-    <row r="519" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="519" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W519" s="7"/>
     </row>
-    <row r="520" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="520" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W520" s="7"/>
     </row>
-    <row r="521" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="521" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W521" s="7"/>
     </row>
-    <row r="522" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="522" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W522" s="7"/>
     </row>
-    <row r="523" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="523" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W523" s="7"/>
     </row>
-    <row r="524" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="524" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W524" s="7"/>
     </row>
-    <row r="525" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="525" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W525" s="7"/>
     </row>
-    <row r="526" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="526" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W526" s="7"/>
     </row>
-    <row r="527" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="527" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W527" s="7"/>
     </row>
-    <row r="528" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="528" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W528" s="7"/>
     </row>
-    <row r="529" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="529" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W529" s="7"/>
     </row>
-    <row r="530" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="530" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W530" s="7"/>
     </row>
-    <row r="531" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="531" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W531" s="7"/>
     </row>
-    <row r="532" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="532" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W532" s="7"/>
     </row>
-    <row r="533" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="533" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W533" s="7"/>
     </row>
-    <row r="534" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="534" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W534" s="7"/>
     </row>
-    <row r="535" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="535" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W535" s="7"/>
     </row>
-    <row r="536" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="536" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W536" s="7"/>
     </row>
-    <row r="537" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="537" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W537" s="7"/>
     </row>
-    <row r="538" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="538" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W538" s="7"/>
     </row>
-    <row r="539" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="539" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W539" s="7"/>
     </row>
-    <row r="540" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="540" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W540" s="7"/>
     </row>
-    <row r="541" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="541" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W541" s="7"/>
     </row>
-    <row r="542" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="542" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W542" s="7"/>
     </row>
-    <row r="543" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="543" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W543" s="7"/>
     </row>
-    <row r="544" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="544" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W544" s="7"/>
     </row>
-    <row r="545" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="545" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W545" s="7"/>
     </row>
-    <row r="546" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="546" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W546" s="7"/>
     </row>
-    <row r="547" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="547" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W547" s="7"/>
     </row>
-    <row r="548" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="548" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W548" s="7"/>
     </row>
-    <row r="549" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="549" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W549" s="7"/>
     </row>
-    <row r="550" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="550" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W550" s="7"/>
     </row>
-    <row r="551" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="551" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W551" s="7"/>
     </row>
-    <row r="552" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="552" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W552" s="7"/>
     </row>
-    <row r="553" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="553" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W553" s="7"/>
     </row>
-    <row r="554" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="554" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W554" s="7"/>
     </row>
-    <row r="555" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="555" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W555" s="7"/>
     </row>
-    <row r="556" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="556" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W556" s="7"/>
     </row>
-    <row r="557" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="557" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W557" s="7"/>
     </row>
-    <row r="558" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="558" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W558" s="7"/>
     </row>
-    <row r="559" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="559" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W559" s="7"/>
     </row>
-    <row r="560" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="560" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W560" s="7"/>
     </row>
-    <row r="561" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="561" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W561" s="7"/>
     </row>
-    <row r="562" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="562" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W562" s="7"/>
     </row>
-    <row r="563" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="563" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W563" s="7"/>
     </row>
-    <row r="564" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="564" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W564" s="7"/>
     </row>
-    <row r="565" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="565" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W565" s="7"/>
     </row>
-    <row r="566" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="566" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W566" s="7"/>
     </row>
-    <row r="567" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="567" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W567" s="7"/>
     </row>
-    <row r="568" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="568" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W568" s="7"/>
     </row>
-    <row r="569" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="569" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W569" s="7"/>
     </row>
-    <row r="570" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="570" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W570" s="7"/>
     </row>
-    <row r="571" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W571" s="7"/>
     </row>
-    <row r="572" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="572" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W572" s="7"/>
     </row>
-    <row r="573" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="573" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W573" s="7"/>
     </row>
-    <row r="574" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W574" s="7"/>
     </row>
-    <row r="575" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="575" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W575" s="7"/>
     </row>
-    <row r="576" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="576" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W576" s="7"/>
     </row>
-    <row r="577" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W577" s="7"/>
     </row>
-    <row r="578" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="578" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W578" s="7"/>
     </row>
-    <row r="579" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="579" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W579" s="7"/>
     </row>
-    <row r="580" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="580" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W580" s="7"/>
     </row>
-    <row r="581" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W581" s="7"/>
     </row>
-    <row r="582" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="582" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W582" s="7"/>
     </row>
-    <row r="583" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="583" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W583" s="7"/>
     </row>
-    <row r="584" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="584" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W584" s="7"/>
     </row>
-    <row r="585" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="585" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W585" s="7"/>
     </row>
-    <row r="586" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="586" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W586" s="7"/>
     </row>
-    <row r="587" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="587" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W587" s="7"/>
     </row>
-    <row r="588" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="588" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W588" s="7"/>
     </row>
-    <row r="589" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="589" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W589" s="7"/>
     </row>
-    <row r="590" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="590" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W590" s="7"/>
     </row>
-    <row r="591" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="591" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W591" s="7"/>
     </row>
-    <row r="592" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="592" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W592" s="7"/>
     </row>
-    <row r="593" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="593" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W593" s="7"/>
     </row>
-    <row r="594" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="594" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W594" s="7"/>
     </row>
-    <row r="595" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="595" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W595" s="7"/>
     </row>
-    <row r="596" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="596" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W596" s="7"/>
     </row>
-    <row r="597" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="597" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W597" s="7"/>
     </row>
-    <row r="598" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="598" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W598" s="7"/>
     </row>
-    <row r="599" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="599" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W599" s="7"/>
     </row>
-    <row r="600" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="600" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W600" s="7"/>
     </row>
-    <row r="601" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="601" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W601" s="7"/>
     </row>
-    <row r="602" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="602" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W602" s="7"/>
     </row>
-    <row r="603" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="603" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W603" s="7"/>
     </row>
-    <row r="604" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="604" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W604" s="7"/>
     </row>
-    <row r="605" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="605" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W605" s="7"/>
     </row>
-    <row r="606" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="606" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W606" s="7"/>
     </row>
-    <row r="607" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="607" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W607" s="7"/>
     </row>
-    <row r="608" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="608" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W608" s="7"/>
     </row>
-    <row r="609" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="609" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W609" s="7"/>
     </row>
-    <row r="610" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="610" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W610" s="7"/>
     </row>
-    <row r="611" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="611" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W611" s="7"/>
     </row>
-    <row r="612" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="612" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W612" s="7"/>
     </row>
-    <row r="613" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="613" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W613" s="7"/>
     </row>
-    <row r="614" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="614" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W614" s="7"/>
     </row>
-    <row r="615" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="615" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W615" s="7"/>
     </row>
-    <row r="616" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="616" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W616" s="7"/>
     </row>
-    <row r="617" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="617" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W617" s="7"/>
     </row>
-    <row r="618" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="618" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W618" s="7"/>
     </row>
-    <row r="619" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="619" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W619" s="7"/>
     </row>
-    <row r="620" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="620" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W620" s="7"/>
     </row>
-    <row r="621" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="621" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W621" s="7"/>
     </row>
-    <row r="622" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="622" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W622" s="7"/>
     </row>
-    <row r="623" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="623" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W623" s="7"/>
     </row>
-    <row r="624" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="624" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W624" s="7"/>
     </row>
-    <row r="625" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="625" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W625" s="7"/>
     </row>
-    <row r="626" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="626" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W626" s="7"/>
     </row>
-    <row r="627" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="627" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W627" s="7"/>
     </row>
-    <row r="628" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="628" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W628" s="7"/>
     </row>
-    <row r="629" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="629" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W629" s="7"/>
     </row>
-    <row r="630" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="630" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W630" s="7"/>
     </row>
-    <row r="631" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="631" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W631" s="7"/>
     </row>
-    <row r="632" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="632" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W632" s="7"/>
     </row>
-    <row r="633" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="633" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W633" s="7"/>
     </row>
-    <row r="634" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="634" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W634" s="7"/>
     </row>
-    <row r="635" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="635" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W635" s="7"/>
     </row>
-    <row r="636" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="636" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W636" s="7"/>
     </row>
-    <row r="637" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="637" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W637" s="7"/>
     </row>
-    <row r="638" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="638" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W638" s="7"/>
     </row>
-    <row r="639" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="639" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W639" s="7"/>
     </row>
-    <row r="640" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="640" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W640" s="7"/>
     </row>
-    <row r="641" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="641" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W641" s="7"/>
     </row>
-    <row r="642" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="642" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W642" s="7"/>
     </row>
-    <row r="643" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="643" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W643" s="7"/>
     </row>
-    <row r="644" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="644" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W644" s="7"/>
     </row>
-    <row r="645" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="645" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W645" s="7"/>
     </row>
-    <row r="646" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="646" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W646" s="7"/>
     </row>
-    <row r="647" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="647" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W647" s="7"/>
     </row>
-    <row r="648" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="648" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W648" s="7"/>
     </row>
-    <row r="649" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="649" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W649" s="7"/>
     </row>
-    <row r="650" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="650" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W650" s="7"/>
     </row>
-    <row r="651" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="651" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W651" s="7"/>
     </row>
-    <row r="652" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="652" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W652" s="7"/>
     </row>
-    <row r="653" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="653" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W653" s="7"/>
     </row>
-    <row r="654" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="654" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W654" s="7"/>
     </row>
-    <row r="655" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="655" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W655" s="7"/>
     </row>
-    <row r="656" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="656" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W656" s="7"/>
     </row>
-    <row r="657" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="657" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W657" s="7"/>
     </row>
-    <row r="658" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="658" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W658" s="7"/>
     </row>
-    <row r="659" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="659" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W659" s="7"/>
     </row>
-    <row r="660" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="660" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W660" s="7"/>
     </row>
-    <row r="661" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="661" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W661" s="7"/>
     </row>
-    <row r="662" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="662" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W662" s="7"/>
     </row>
-    <row r="663" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="663" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W663" s="7"/>
     </row>
-    <row r="664" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="664" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W664" s="7"/>
     </row>
-    <row r="665" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="665" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W665" s="7"/>
     </row>
-    <row r="666" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="666" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W666" s="7"/>
     </row>
-    <row r="667" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="667" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W667" s="7"/>
     </row>
-    <row r="668" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="668" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W668" s="7"/>
     </row>
-    <row r="669" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="669" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W669" s="7"/>
     </row>
-    <row r="670" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="670" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W670" s="7"/>
     </row>
-    <row r="671" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="671" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W671" s="7"/>
     </row>
-    <row r="672" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="672" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W672" s="7"/>
     </row>
-    <row r="673" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="673" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W673" s="7"/>
     </row>
-    <row r="674" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="674" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W674" s="7"/>
     </row>
-    <row r="675" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="675" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W675" s="7"/>
     </row>
-    <row r="676" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="676" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W676" s="7"/>
     </row>
-    <row r="677" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="677" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W677" s="7"/>
     </row>
-    <row r="678" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="678" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W678" s="7"/>
     </row>
-    <row r="679" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="679" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W679" s="7"/>
     </row>
-    <row r="680" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="680" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W680" s="7"/>
     </row>
-    <row r="681" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="681" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W681" s="7"/>
     </row>
-    <row r="682" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="682" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W682" s="7"/>
     </row>
-    <row r="683" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="683" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W683" s="7"/>
     </row>
-    <row r="684" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="684" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W684" s="7"/>
     </row>
-    <row r="685" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="685" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W685" s="7"/>
     </row>
-    <row r="686" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="686" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W686" s="7"/>
     </row>
-    <row r="687" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="687" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W687" s="7"/>
     </row>
-    <row r="688" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="688" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W688" s="7"/>
     </row>
-    <row r="689" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="689" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W689" s="7"/>
     </row>
-    <row r="690" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="690" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W690" s="7"/>
     </row>
-    <row r="691" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="691" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W691" s="7"/>
     </row>
-    <row r="692" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="692" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W692" s="7"/>
     </row>
-    <row r="693" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="693" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W693" s="7"/>
     </row>
-    <row r="694" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="694" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W694" s="7"/>
     </row>
-    <row r="695" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="695" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W695" s="7"/>
     </row>
-    <row r="696" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="696" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W696" s="7"/>
     </row>
-    <row r="697" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="697" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W697" s="7"/>
     </row>
-    <row r="698" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="698" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W698" s="7"/>
     </row>
-    <row r="699" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="699" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W699" s="7"/>
     </row>
-    <row r="700" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="700" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W700" s="7"/>
     </row>
-    <row r="701" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="701" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W701" s="7"/>
     </row>
-    <row r="702" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="702" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W702" s="7"/>
     </row>
-    <row r="703" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="703" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W703" s="7"/>
     </row>
-    <row r="704" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="704" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W704" s="7"/>
     </row>
-    <row r="705" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="705" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W705" s="7"/>
     </row>
-    <row r="706" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="706" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W706" s="7"/>
     </row>
-    <row r="707" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="707" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W707" s="7"/>
     </row>
-    <row r="708" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="708" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W708" s="7"/>
     </row>
-    <row r="709" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="709" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W709" s="7"/>
     </row>
-    <row r="710" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="710" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W710" s="7"/>
     </row>
-    <row r="711" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="711" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W711" s="7"/>
     </row>
-    <row r="712" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="712" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W712" s="7"/>
     </row>
-    <row r="713" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="713" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W713" s="7"/>
     </row>
-    <row r="714" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="714" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W714" s="7"/>
     </row>
-    <row r="715" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="715" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W715" s="7"/>
     </row>
-    <row r="716" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="716" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W716" s="7"/>
     </row>
-    <row r="717" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="717" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W717" s="7"/>
     </row>
-    <row r="718" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="718" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W718" s="7"/>
     </row>
-    <row r="719" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="719" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W719" s="7"/>
     </row>
-    <row r="720" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="720" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W720" s="7"/>
     </row>
-    <row r="721" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="721" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W721" s="7"/>
     </row>
-    <row r="722" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="722" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W722" s="7"/>
     </row>
-    <row r="723" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="723" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W723" s="7"/>
     </row>
-    <row r="724" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="724" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W724" s="7"/>
     </row>
-    <row r="725" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="725" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W725" s="7"/>
     </row>
-    <row r="726" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="726" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W726" s="7"/>
     </row>
-    <row r="727" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="727" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W727" s="7"/>
     </row>
-    <row r="728" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="728" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W728" s="7"/>
     </row>
-    <row r="729" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="729" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W729" s="7"/>
     </row>
-    <row r="730" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="730" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W730" s="7"/>
     </row>
-    <row r="731" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="731" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W731" s="7"/>
     </row>
-    <row r="732" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="732" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W732" s="7"/>
     </row>
-    <row r="733" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="733" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W733" s="7"/>
     </row>
-    <row r="734" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="734" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W734" s="7"/>
     </row>
-    <row r="735" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="735" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W735" s="7"/>
     </row>
-    <row r="736" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="736" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W736" s="7"/>
     </row>
-    <row r="737" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="737" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W737" s="7"/>
     </row>
-    <row r="738" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="738" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W738" s="7"/>
     </row>
-    <row r="739" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="739" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W739" s="7"/>
     </row>
-    <row r="740" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="740" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W740" s="7"/>
     </row>
-    <row r="741" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="741" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W741" s="7"/>
     </row>
-    <row r="742" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="742" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W742" s="7"/>
     </row>
-    <row r="743" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="743" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W743" s="7"/>
     </row>
-    <row r="744" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="744" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W744" s="7"/>
     </row>
-    <row r="745" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="745" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25">
       <c r="W745" s="7"/>
     </row>
-    <row r="746" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="747" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="748" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="749" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="750" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25"/>
+    <row r="747" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25"/>
+    <row r="748" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25"/>
+    <row r="749" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25"/>
+    <row r="750" spans="23:23" ht="14.25" customHeight="1" ns3:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <autoFilter ref="A9:W193" ns2:uid="{00000000-0001-0000-0200-000000000000}">
     <filterColumn colId="2">
       <filters>
         <filter val="PSS"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:W193">
+    <sortState ref="A10:W193">
       <sortCondition ref="A9:A190"/>
     </sortState>
   </autoFilter>
@@ -15049,30 +15052,30 @@
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" ns4:id="rId1"/>
+  <legacyDrawing ns4:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
-          <x14:formula1>
-            <xm:f>Sheet1!$B$2:$B$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>M10:N193 P10:R193 J10:J193</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
-          <x14:formula1>
-            <xm:f>Sheet1!$A$2:$A$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>T10:T193</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3DE61C5E-9DA3-4CE3-A1FF-8FBE651EA6B5}">
-          <x14:formula1>
-            <xm:f>'LISTA VALORI'!$A$2:$A$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>K10:K193</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns5:dataValidations count="3">
+        <ns5:dataValidation type="list" allowBlank="1" showErrorMessage="1" ns2:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
+          <ns5:formula1>
+            <ns6:f>Sheet1!$B$2:$B$3</ns6:f>
+          </ns5:formula1>
+          <ns6:sqref>M10:N193 P10:R193 J10:J193</ns6:sqref>
+        </ns5:dataValidation>
+        <ns5:dataValidation type="list" allowBlank="1" showErrorMessage="1" ns2:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
+          <ns5:formula1>
+            <ns6:f>Sheet1!$A$2:$A$3</ns6:f>
+          </ns5:formula1>
+          <ns6:sqref>T10:T193</ns6:sqref>
+        </ns5:dataValidation>
+        <ns5:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" ns2:uid="{3DE61C5E-9DA3-4CE3-A1FF-8FBE651EA6B5}">
+          <ns5:formula1>
+            <ns6:f>'LISTA VALORI'!$A$2:$A$8</ns6:f>
+          </ns5:formula1>
+          <ns6:sqref>K10:K193</ns6:sqref>
+        </ns5:dataValidation>
+      </ns5:dataValidations>
     </ext>
   </extLst>
 </worksheet>

</xml_diff>